<commit_message>
feat: validate min paying guests, dietary preferences, and unified provider service requests
</commit_message>
<xml_diff>
--- a/Mau_Danh_Sach_Khach_Tour_TC-9901.xlsx
+++ b/Mau_Danh_Sach_Khach_Tour_TC-9901.xlsx
@@ -64,8 +64,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,15 +398,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I5"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
     <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="26.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="45.83203125" customWidth="1"/>
+    <col min="8" max="8" width="40.83203125" customWidth="1"/>
+    <col min="9" max="9" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,7 +431,13 @@
         <v>Loại khách</v>
       </c>
       <c r="G1" t="str">
-        <v>Ghi chú</v>
+        <v>Nguyện vọng xếp phòng / Muốn ở cùng ai</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Yêu cầu ăn uống / Dị ứng thực phẩm</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Ghi chú cá nhân</v>
       </c>
     </row>
     <row r="2">
@@ -438,7 +447,7 @@
       <c r="B2" t="str">
         <v>Nguyễn Văn An</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C2" s="1" t="str">
         <v>001090012345</v>
       </c>
       <c r="D2" t="str">
@@ -451,7 +460,13 @@
         <v>Người lớn</v>
       </c>
       <c r="G2" t="str">
-        <v>Người đại diện đoàn, ăn chay nhẹ</v>
+        <v>Muốn ở cùng Trần Thị Bình (STT 2), ưu tiên hai giường đơn</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Ăn chay ngày rằm, không ăn cay</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Người đại diện đoàn</v>
       </c>
     </row>
     <row r="3">
@@ -461,7 +476,7 @@
       <c r="B3" t="str">
         <v>Trần Thị Bình</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C3" s="1" t="str">
         <v>001192005678</v>
       </c>
       <c r="D3" t="str">
@@ -474,6 +489,12 @@
         <v>Người lớn</v>
       </c>
       <c r="G3" t="str">
+        <v>Muốn ở cùng Nguyễn Văn An (STT 1)</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Không ăn thịt bò</v>
+      </c>
+      <c r="I3" t="str">
         <v>Hay say xe ngồi đầu xe</v>
       </c>
     </row>
@@ -484,7 +505,7 @@
       <c r="B4" t="str">
         <v>Nguyễn Gia Hưng</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C4" s="1" t="str">
         <v>001218009999</v>
       </c>
       <c r="D4" t="str">
@@ -497,7 +518,13 @@
         <v>Trẻ em (2–11 tuổi)</v>
       </c>
       <c r="G4" t="str">
-        <v>Dị ứng hải sản</v>
+        <v>Ở cùng phòng bố mẹ (Nguyễn Văn An)</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Dị ứng hải sản, tôm cua, kiêng đậu phộng</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Trẻ nhỏ cần chú ý</v>
       </c>
     </row>
     <row r="5">
@@ -507,7 +534,7 @@
       <c r="B5" t="str">
         <v>Nguyễn Bảo Ngọc</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C5" s="1" t="str">
         <v/>
       </c>
       <c r="D5" t="str">
@@ -520,12 +547,18 @@
         <v>Trẻ em (dưới 2 tuổi)</v>
       </c>
       <c r="G5" t="str">
-        <v>Cần nôi / ghế trẻ em</v>
+        <v>Cần nôi trẻ em trong phòng</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Dùng thức ăn mềm / cháo dinh dưỡng</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Em bé cần nôi</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>